<commit_message>
0.6.6 AMBER 99%, paper 95%, web 90%
</commit_message>
<xml_diff>
--- a/DATASET/Hypocreales.xlsx
+++ b/DATASET/Hypocreales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25970" windowHeight="15390"/>
+    <workbookView windowWidth="18350" windowHeight="15980"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>Taxon</t>
   </si>
@@ -133,18 +133,6 @@
     <t>PQ468423</t>
   </si>
   <si>
-    <t xml:space="preserve">Fusarium oxysporum </t>
-  </si>
-  <si>
-    <t>NC_017930</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fusarium solani </t>
-  </si>
-  <si>
-    <t>NC_016680</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hirsutella minnesotensis </t>
   </si>
   <si>
@@ -191,12 +179,6 @@
   </si>
   <si>
     <t>NC_008068</t>
-  </si>
-  <si>
-    <t>Neurospora crassa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> KY498478</t>
   </si>
   <si>
     <t xml:space="preserve">Ophiocordyceps sinensis </t>
@@ -1249,7 +1231,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="28.8181818181818" customWidth="1"/>
@@ -1492,7 +1474,7 @@
       <c r="A30" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="5" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1516,7 +1498,7 @@
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="3" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1534,30 +1516,6 @@
       </c>
       <c r="B35" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
0.6.9 AMBER 99%, paper 97%, web 91%
</commit_message>
<xml_diff>
--- a/DATASET/Hypocreales.xlsx
+++ b/DATASET/Hypocreales.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="15980"/>
+    <workbookView windowWidth="25970" windowHeight="15390"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t>Taxon</t>
   </si>
@@ -133,6 +133,18 @@
     <t>PQ468423</t>
   </si>
   <si>
+    <t xml:space="preserve">Fusarium oxysporum </t>
+  </si>
+  <si>
+    <t>NC_017930</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusarium solani </t>
+  </si>
+  <si>
+    <t>NC_016680</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hirsutella minnesotensis </t>
   </si>
   <si>
@@ -179,6 +191,12 @@
   </si>
   <si>
     <t>NC_008068</t>
+  </si>
+  <si>
+    <t>Neurospora crassa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KY498478</t>
   </si>
   <si>
     <t xml:space="preserve">Ophiocordyceps sinensis </t>
@@ -1231,7 +1249,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="28.8181818181818" customWidth="1"/>
@@ -1474,7 +1492,7 @@
       <c r="A30" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="3" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1498,7 +1516,7 @@
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="5" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1516,6 +1534,30 @@
       </c>
       <c r="B35" s="3" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>